<commit_message>
Update to About page
</commit_message>
<xml_diff>
--- a/InputData/hydgn/BSfHPbP/BAU Subsidy for Hydgn Prod by Pathway.xlsx
+++ b/InputData/hydgn/BSfHPbP/BAU Subsidy for Hydgn Prod by Pathway.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us-analysis\InputData\hydgn\BSfHPbP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\hydgn\BSfHPbP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12EAAC3D-75BA-4EE2-97F9-3DF74D00BB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E74F3C4B-C72E-4F62-AD8D-71E7DDB3ED2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-22170" yWindow="2010" windowWidth="21120" windowHeight="14655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -43,10 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
-  <si>
-    <t>HPEC Hydrogen Production Equipment CapEx</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
   <si>
     <t>Source:</t>
   </si>
@@ -66,18 +63,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>We average the use of the hydrogen plant out over the</t>
-  </si>
-  <si>
-    <t>course of a year to convert between kW and kWh,</t>
-  </si>
-  <si>
-    <t>necessary to convert BTU/yr of hydrogen production</t>
-  </si>
-  <si>
-    <t>capacity to $ of CapEx using the $/kW conversion factor.</t>
-  </si>
-  <si>
     <t>Currency Year</t>
   </si>
   <si>
@@ -136,6 +121,9 @@
   </si>
   <si>
     <t>btu/lb H2</t>
+  </si>
+  <si>
+    <t>BSfHPbP BAU Subsidy for Hydrogen Production by Pathway</t>
   </si>
 </sst>
 </file>
@@ -488,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="45.85546875" customWidth="1"/>
@@ -496,15 +484,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -515,83 +503,63 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>17</v>
+      <c r="A16">
+        <v>0.78452102304761584</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>18</v>
+      <c r="A18" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="7"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>42</v>
+      </c>
+      <c r="B19" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>19</v>
+      <c r="A20">
+        <f>3.41214*10^6</f>
+        <v>3412140</v>
+      </c>
+      <c r="B20" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>0.78452102304761584</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23" s="7"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>42</v>
-      </c>
-      <c r="B24" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <f>3.41214*10^6</f>
-        <v>3412140</v>
-      </c>
-      <c r="B25" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26">
         <v>61013</v>
       </c>
-      <c r="B26" t="s">
-        <v>30</v>
+      <c r="B21" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -611,12 +579,12 @@
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B3">
         <v>3</v>
@@ -624,16 +592,16 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B4">
-        <f>About!A26</f>
+        <f>About!A21</f>
         <v>61013</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B5">
         <v>2.2046199999999998</v>
@@ -641,7 +609,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B6">
         <f>B4*B5</f>
@@ -650,16 +618,16 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B7">
-        <f>B3/B6*About!A21</f>
+        <f>B3/B6*About!A16</f>
         <v>1.7497246817445102E-5</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B9">
         <v>0.75</v>
@@ -667,7 +635,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B10">
         <f>B4</f>
@@ -676,7 +644,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B11">
         <f>B5</f>
@@ -685,7 +653,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B12">
         <f>B10*B11</f>
@@ -694,10 +662,10 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B13">
-        <f>B9/B12*About!A21</f>
+        <f>B9/B12*About!A16</f>
         <v>4.3743117043612755E-6</v>
       </c>
     </row>
@@ -719,7 +687,7 @@
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B1" s="4">
         <v>2021</v>
@@ -814,7 +782,7 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" s="5">
         <v>0</v>
@@ -909,7 +877,7 @@
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="5">
         <v>0</v>
@@ -1004,7 +972,7 @@
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="5">
         <v>0</v>
@@ -1099,7 +1067,7 @@
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" s="5">
         <v>0</v>
@@ -1194,7 +1162,7 @@
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B6" s="5">
         <v>0</v>
@@ -1289,7 +1257,7 @@
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B7" s="5">
         <v>0</v>
@@ -1395,7 +1363,7 @@
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B8" s="5">
         <v>0</v>

</xml_diff>